<commit_message>
fix: remove asterisks from Excel template headers, make normalize_header strip trailing markers
- normalize_header now strips trailing * and other marker chars before slugifying
- Excel templates use color-coded headers (green=required, gray=optional) instead of *
- Verified: nombre*→nombre, rut*→rut, apellidos*→apellidos, correo*→correo
</commit_message>
<xml_diff>
--- a/frontend/public/plantilla_estudiantes.xlsx
+++ b/frontend/public/plantilla_estudiantes.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +41,11 @@
       <sz val="11"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="0094A3B8"/>
+      <sz val="11"/>
+    </font>
+    <font>
       <sz val="10"/>
     </font>
     <font>
@@ -49,7 +54,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -64,8 +69,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A5F"/>
-        <bgColor rgb="001E3A5F"/>
+        <fgColor rgb="00065F46"/>
+        <bgColor rgb="00065F46"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0064748B"/>
+        <bgColor rgb="0064748B"/>
       </patternFill>
     </fill>
     <fill>
@@ -101,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -110,9 +121,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -500,241 +514,241 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Completa las columnas con los datos de cada estudiante. La fila 5 es la primera de ejemplo. Los campos con * son obligatorios.</t>
+          <t>Completa una fila por cada estudiante. Los encabezados en VERDE OSCURO son obligatorios, los GRISES son opcionales. La fila 5 es un ejemplo.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>El Numero ECOE se asigna automaticamente (no es necesario llenarlo). El correo debe corresponder a un usuario con rol 'estudiante' ya registrado.</t>
+          <t>El Numero ECOE se asigna automaticamente (puedes dejarlo vacio o borrar la columna). El correo no requiere cuenta de usuario en el sistema.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>nombre*</t>
+          <t>nombre</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>apellidos*</t>
+          <t>apellidos</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>rut*</t>
+          <t>rut</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>correo*</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+          <t>correo</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>numero_ecoe</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>grupo</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>circuito</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Ana</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Perez Gonzalez</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>11111111-1</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>ana.perez@ejemplo.cl</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>(automatico)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Grupo 1</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Circuito A</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Bruno</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Soto Morales</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>22222222-2</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>bruno.soto@ejemplo.cl</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>(automatico)</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Grupo 1</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Circuito A</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Camila</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Rojas Vega</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>33333333-3</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>camila.rojas@ejemplo.cl</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>(automatico)</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Grupo 2</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Circuito B</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Diego</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Munoz Castillo</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>44444444-4</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>diego.munoz@ejemplo.cl</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>(automatico)</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Grupo 2</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Circuito B</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Elena</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Flores Rivas</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>55555555-5</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>elena.flores@ejemplo.cl</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>(automatico)</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Grupo 3</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Circuito A</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Elimina las filas de ejemplo antes de importar. Guarda como .xlsx o .csv (UTF-8).</t>
         </is>

</xml_diff>

<commit_message>
fix: move Excel template headers to row 1, instructions on separate sheet
- Headers now on row 1 (not row 4), so pandas reads them directly
- Instructions moved to a separate 'Instrucciones' sheet
- Required columns in green, optional in gray — no asterisks
- Verified: pandas reads nombre, apellidos, rut, correo correctly
</commit_message>
<xml_diff>
--- a/frontend/public/plantilla_estudiantes.xlsx
+++ b/frontend/public/plantilla_estudiantes.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Estudiantes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,45 +28,32 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001E3A5F"/>
-      <sz val="13"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="001E40AF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0094A3B8"/>
+      <color rgb="0064748B"/>
       <sz val="11"/>
     </font>
     <font>
       <sz val="10"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="0094A3B8"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="001E3A5F"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F0FE"/>
-        <bgColor rgb="00E8F0FE"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -112,21 +100,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -507,260 +492,289 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PLANTILLA PARA CARGA MASIVA DE ESTUDIANTES - ECOE</t>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>apellidos</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>rut</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>correo</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>numero_ecoe</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>grupo</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>circuito</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Completa una fila por cada estudiante. Los encabezados en VERDE OSCURO son obligatorios, los GRISES son opcionales. La fila 5 es un ejemplo.</t>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Ana</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Perez Gonzalez</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>11111111-1</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>ana.perez@ejemplo.cl</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Grupo 1</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Circuito A</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>El Numero ECOE se asigna automaticamente (puedes dejarlo vacio o borrar la columna). El correo no requiere cuenta de usuario en el sistema.</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Bruno</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Soto Morales</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>22222222-2</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>bruno.soto@ejemplo.cl</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Grupo 1</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Circuito A</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>nombre</t>
+          <t>Camila</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>apellidos</t>
+          <t>Rojas Vega</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>rut</t>
+          <t>33333333-3</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>correo</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>numero_ecoe</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>grupo</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>circuito</t>
+          <t>camila.rojas@ejemplo.cl</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Grupo 2</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Circuito B</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Ana</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Perez Gonzalez</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>11111111-1</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>ana.perez@ejemplo.cl</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>(automatico)</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Grupo 1</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Munoz Castillo</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>44444444-4</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>diego.munoz@ejemplo.cl</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Grupo 2</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Circuito B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Elena</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Flores Rivas</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>55555555-5</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>elena.flores@ejemplo.cl</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Grupo 3</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Circuito A</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Como usar esta plantilla</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>1. La pestana 'Estudiantes' tiene los encabezados en la FILA 1. No agregues filas antes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>2. Completa una fila por cada estudiante a partir de la fila 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>3. Encabezados VERDE OSCURO = obligatorios. Encabezados GRIS = opcionales.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Bruno</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Soto Morales</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>22222222-2</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>bruno.soto@ejemplo.cl</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>(automatico)</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Grupo 1</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Circuito A</t>
+          <t>4. Campos obligatorios: nombre, apellidos, rut, correo.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Camila</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Rojas Vega</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>33333333-3</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>camila.rojas@ejemplo.cl</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>(automatico)</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Grupo 2</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Circuito B</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>5. El Numero ECOE se asigna automaticamente. Dejalo vacio.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Diego</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Munoz Castillo</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>44444444-4</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>diego.munoz@ejemplo.cl</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>(automatico)</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Grupo 2</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Circuito B</t>
+          <t>6. El correo es el email del estudiante. NO necesita cuenta de usuario en el sistema.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Elena</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Flores Rivas</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>55555555-5</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>elena.flores@ejemplo.cl</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>(automatico)</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Grupo 3</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Circuito A</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>7. Elimina las filas de ejemplo antes de importar.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>Elimina las filas de ejemplo antes de importar. Guarda como .xlsx o .csv (UTF-8).</t>
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>8. Guarda como .xlsx o .csv (UTF-8) y subelo en la pagina de Estudiantes.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A10:G10"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>